<commit_message>
Remove obsolete Excel files and update error handling in artikelnummern.py. The input.xlsx and 260703-masterdatei.xlsx files have been deleted to streamline project resources. Additionally, the error handling in artikelnummern.py has been improved to provide clearer messages regarding resolution errors.
</commit_message>
<xml_diff>
--- a/data/gruppen.xlsx
+++ b/data/gruppen.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10329"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/kristinkolloff/Dropbox/PPROSEMA/weclapp/Import/source-files/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/chris-mbp/switchdrive/ext/prosema/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4D5673C3-D3E1-1D44-924E-09B4D6DBDF63}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E1206DBD-B420-C545-9417-71D3CAF5D22C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="600" windowWidth="28800" windowHeight="15820" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="600" windowWidth="28800" windowHeight="15820" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Anleitung" sheetId="1" r:id="rId1"/>
@@ -468,13 +468,13 @@
     <t>Taktile Noppenmatten</t>
   </si>
   <si>
-    <t>Takktile Einzelrippen</t>
-  </si>
-  <si>
     <t>Taktile Rippenfolien</t>
   </si>
   <si>
     <t>Abschlussprofile Messing</t>
+  </si>
+  <si>
+    <t>Taktile Einzelrippen</t>
   </si>
 </sst>
 </file>
@@ -584,7 +584,7 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Standard" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
@@ -1268,7 +1268,7 @@
         <v>28</v>
       </c>
       <c r="C11" s="6" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="D11" s="7" t="s">
         <v>63</v>
@@ -1786,7 +1786,7 @@
         <v>24</v>
       </c>
       <c r="C48" s="6" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="D48" s="7" t="s">
         <v>133</v>
@@ -1800,7 +1800,7 @@
         <v>26</v>
       </c>
       <c r="C49" s="6" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="D49" s="7" t="s">
         <v>134</v>

</xml_diff>